<commit_message>
[FixDev]: fix pydantic paths for extract and transform modules
</commit_message>
<xml_diff>
--- a/frontend/web/app/analisis_frecuencia_discrepancia_combustible.xlsx
+++ b/frontend/web/app/analisis_frecuencia_discrepancia_combustible.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Develop\FuelOptiMine\frontend\web\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AC5F59-9C77-4044-942C-627529398FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A6F45F-7390-40BB-A9E2-DA0EE1C1A4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{7CCE9A0B-2825-43BC-B7A8-B67F7FB503E1}"/>
   </bookViews>
@@ -1406,7 +1406,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1415,24 +1415,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="34" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="0" fillId="34" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3005,6 +3001,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1938343135"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -8558,10 +8555,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="6"/>
+      <c r="B1" s="9"/>
       <c r="C1" s="4" t="s">
         <v>14</v>
       </c>
@@ -8855,126 +8852,126 @@
       <c r="F14" s="1"/>
     </row>
     <row r="29" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q29" s="7" t="s">
+      <c r="Q29" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="R29" s="6"/>
-      <c r="S29" s="6"/>
-      <c r="T29" s="6"/>
-      <c r="U29" s="6"/>
-      <c r="V29" s="6"/>
-      <c r="W29" s="6"/>
-      <c r="X29" s="6"/>
-      <c r="Y29" s="6"/>
-      <c r="Z29" s="6"/>
+      <c r="R29" s="9"/>
+      <c r="S29" s="9"/>
+      <c r="T29" s="9"/>
+      <c r="U29" s="9"/>
+      <c r="V29" s="9"/>
+      <c r="W29" s="9"/>
+      <c r="X29" s="9"/>
+      <c r="Y29" s="9"/>
+      <c r="Z29" s="9"/>
     </row>
     <row r="30" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
-      <c r="T30" s="6"/>
-      <c r="U30" s="6"/>
-      <c r="V30" s="6"/>
-      <c r="W30" s="6"/>
-      <c r="X30" s="6"/>
-      <c r="Y30" s="6"/>
-      <c r="Z30" s="6"/>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9"/>
+      <c r="S30" s="9"/>
+      <c r="T30" s="9"/>
+      <c r="U30" s="9"/>
+      <c r="V30" s="9"/>
+      <c r="W30" s="9"/>
+      <c r="X30" s="9"/>
+      <c r="Y30" s="9"/>
+      <c r="Z30" s="9"/>
     </row>
     <row r="31" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q31" s="6"/>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
-      <c r="T31" s="6"/>
-      <c r="U31" s="6"/>
-      <c r="V31" s="6"/>
-      <c r="W31" s="6"/>
-      <c r="X31" s="6"/>
-      <c r="Y31" s="6"/>
-      <c r="Z31" s="6"/>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9"/>
+      <c r="S31" s="9"/>
+      <c r="T31" s="9"/>
+      <c r="U31" s="9"/>
+      <c r="V31" s="9"/>
+      <c r="W31" s="9"/>
+      <c r="X31" s="9"/>
+      <c r="Y31" s="9"/>
+      <c r="Z31" s="9"/>
     </row>
     <row r="32" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q32" s="6"/>
-      <c r="R32" s="6"/>
-      <c r="S32" s="6"/>
-      <c r="T32" s="6"/>
-      <c r="U32" s="6"/>
-      <c r="V32" s="6"/>
-      <c r="W32" s="6"/>
-      <c r="X32" s="6"/>
-      <c r="Y32" s="6"/>
-      <c r="Z32" s="6"/>
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9"/>
+      <c r="S32" s="9"/>
+      <c r="T32" s="9"/>
+      <c r="U32" s="9"/>
+      <c r="V32" s="9"/>
+      <c r="W32" s="9"/>
+      <c r="X32" s="9"/>
+      <c r="Y32" s="9"/>
+      <c r="Z32" s="9"/>
     </row>
     <row r="33" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q33" s="6"/>
-      <c r="R33" s="6"/>
-      <c r="S33" s="6"/>
-      <c r="T33" s="6"/>
-      <c r="U33" s="6"/>
-      <c r="V33" s="6"/>
-      <c r="W33" s="6"/>
-      <c r="X33" s="6"/>
-      <c r="Y33" s="6"/>
-      <c r="Z33" s="6"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
     </row>
     <row r="34" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q34" s="6"/>
-      <c r="R34" s="6"/>
-      <c r="S34" s="6"/>
-      <c r="T34" s="6"/>
-      <c r="U34" s="6"/>
-      <c r="V34" s="6"/>
-      <c r="W34" s="6"/>
-      <c r="X34" s="6"/>
-      <c r="Y34" s="6"/>
-      <c r="Z34" s="6"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
     </row>
     <row r="35" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q35" s="6"/>
-      <c r="R35" s="6"/>
-      <c r="S35" s="6"/>
-      <c r="T35" s="6"/>
-      <c r="U35" s="6"/>
-      <c r="V35" s="6"/>
-      <c r="W35" s="6"/>
-      <c r="X35" s="6"/>
-      <c r="Y35" s="6"/>
-      <c r="Z35" s="6"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
     </row>
     <row r="36" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q36" s="6"/>
-      <c r="R36" s="6"/>
-      <c r="S36" s="6"/>
-      <c r="T36" s="6"/>
-      <c r="U36" s="6"/>
-      <c r="V36" s="6"/>
-      <c r="W36" s="6"/>
-      <c r="X36" s="6"/>
-      <c r="Y36" s="6"/>
-      <c r="Z36" s="6"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
     </row>
     <row r="37" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q37" s="6"/>
-      <c r="R37" s="6"/>
-      <c r="S37" s="6"/>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
-      <c r="V37" s="6"/>
-      <c r="W37" s="6"/>
-      <c r="X37" s="6"/>
-      <c r="Y37" s="6"/>
-      <c r="Z37" s="6"/>
+      <c r="Q37" s="9"/>
+      <c r="R37" s="9"/>
+      <c r="S37" s="9"/>
+      <c r="T37" s="9"/>
+      <c r="U37" s="9"/>
+      <c r="V37" s="9"/>
+      <c r="W37" s="9"/>
+      <c r="X37" s="9"/>
+      <c r="Y37" s="9"/>
+      <c r="Z37" s="9"/>
     </row>
     <row r="38" spans="17:26" x14ac:dyDescent="0.3">
-      <c r="Q38" s="6"/>
-      <c r="R38" s="6"/>
-      <c r="S38" s="6"/>
-      <c r="T38" s="6"/>
-      <c r="U38" s="6"/>
-      <c r="V38" s="6"/>
-      <c r="W38" s="6"/>
-      <c r="X38" s="6"/>
-      <c r="Y38" s="6"/>
-      <c r="Z38" s="6"/>
+      <c r="Q38" s="9"/>
+      <c r="R38" s="9"/>
+      <c r="S38" s="9"/>
+      <c r="T38" s="9"/>
+      <c r="U38" s="9"/>
+      <c r="V38" s="9"/>
+      <c r="W38" s="9"/>
+      <c r="X38" s="9"/>
+      <c r="Y38" s="9"/>
+      <c r="Z38" s="9"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:C11">
@@ -9137,7 +9134,7 @@
         <v>27507</v>
       </c>
       <c r="I7">
-        <f t="shared" ref="I5:I12" si="0">H7+$E$7</f>
+        <f t="shared" ref="I7:I12" si="0">H7+$E$7</f>
         <v>34377.5</v>
       </c>
     </row>
@@ -9149,7 +9146,7 @@
         <v>6</v>
       </c>
       <c r="H8">
-        <f t="shared" ref="H5:H12" si="1">I7</f>
+        <f t="shared" ref="H8" si="1">I7</f>
         <v>34377.5</v>
       </c>
       <c r="I8">
@@ -10627,296 +10624,296 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="11" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="12">
+      <c r="A2" s="7">
         <v>25</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="7">
         <v>6895.5</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="7">
         <f>(A2+B2)/2</f>
         <v>3460.25</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="7">
         <v>76</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="7">
         <f>D2</f>
         <v>76</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="8">
         <f>D2/$E$11</f>
         <v>0.26297577854671278</v>
       </c>
-      <c r="G2" s="15">
+      <c r="G2" s="8">
         <v>0.26297577854671278</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="12">
+      <c r="A3" s="7">
         <v>6895.5</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="7">
         <v>13766</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="7">
         <f t="shared" ref="C3:C11" si="0">(A3+B3)/2</f>
         <v>10330.75</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="7">
         <v>55</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="7">
         <f>D3+E2</f>
         <v>131</v>
       </c>
-      <c r="F3" s="15">
+      <c r="F3" s="8">
         <f t="shared" ref="F3:F11" si="1">D3/$E$11</f>
         <v>0.19031141868512111</v>
       </c>
-      <c r="G3" s="15">
+      <c r="G3" s="8">
         <v>0.45328719723183392</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12">
+      <c r="A4" s="7">
         <v>13766</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="7">
         <v>20636.5</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="7">
         <f t="shared" si="0"/>
         <v>17201.25</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="7">
         <v>21</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="7">
         <f t="shared" ref="E4:E11" si="2">D4+E3</f>
         <v>152</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="8">
         <f t="shared" si="1"/>
         <v>7.2664359861591699E-2</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="8">
         <v>0.52595155709342556</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="12">
+      <c r="A5" s="7">
         <v>20636.5</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="7">
         <v>27507</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="7">
         <f t="shared" si="0"/>
         <v>24071.75</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="7">
         <v>32</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="7">
         <f t="shared" si="2"/>
         <v>184</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="8">
         <f t="shared" si="1"/>
         <v>0.11072664359861592</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="8">
         <v>0.63667820069204151</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="12">
+      <c r="A6" s="7">
         <v>27507</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="7">
         <v>34377.5</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="7">
         <f t="shared" si="0"/>
         <v>30942.25</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="7">
         <v>30</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="7">
         <f t="shared" si="2"/>
         <v>214</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="8">
         <f t="shared" si="1"/>
         <v>0.10380622837370242</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="8">
         <v>0.74048442906574397</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="12">
+      <c r="A7" s="7">
         <v>34377.5</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="7">
         <v>41248</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="7">
         <f t="shared" si="0"/>
         <v>37812.75</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="7">
         <v>20</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="7">
         <f t="shared" si="2"/>
         <v>234</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="8">
         <f t="shared" si="1"/>
         <v>6.9204152249134954E-2</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="8">
         <v>0.80968858131487886</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="12">
+      <c r="A8" s="7">
         <v>41248</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="7">
         <v>48118.5</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="7">
         <f t="shared" si="0"/>
         <v>44683.25</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="7">
         <v>2</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="7">
         <f t="shared" si="2"/>
         <v>236</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="8">
         <f t="shared" si="1"/>
         <v>6.920415224913495E-3</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="8">
         <v>0.81660899653979235</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="12">
+      <c r="A9" s="7">
         <v>48118.5</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="7">
         <v>54989</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="7">
         <f t="shared" si="0"/>
         <v>51553.75</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="7">
         <v>19</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="7">
         <f t="shared" si="2"/>
         <v>255</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="8">
         <f t="shared" si="1"/>
         <v>6.5743944636678195E-2</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="8">
         <v>0.88235294117647056</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="12">
+      <c r="A10" s="7">
         <v>54989</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="7">
         <v>61859.5</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="7">
         <f t="shared" si="0"/>
         <v>58424.25</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="7">
         <v>22</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="7">
         <f t="shared" si="2"/>
         <v>277</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="8">
         <f t="shared" si="1"/>
         <v>7.6124567474048443E-2</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="8">
         <v>0.95847750865051906</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="12">
+      <c r="A11" s="7">
         <v>61859.5</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="7">
         <v>68730</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="7">
         <f t="shared" si="0"/>
         <v>65294.75</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="7">
         <v>12</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="7">
         <f t="shared" si="2"/>
         <v>289</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="8">
         <f t="shared" si="1"/>
         <v>4.1522491349480967E-2</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="2">
         <v>0</v>
       </c>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="9">
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="3">
         <v>1</v>
       </c>
     </row>

</xml_diff>